<commit_message>
Update attendance and dashboards
</commit_message>
<xml_diff>
--- a/frontend/mock_students.xlsx
+++ b/frontend/mock_students.xlsx
@@ -397,62 +397,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Roll No</v>
+      </c>
+      <c r="B1" t="str">
         <v>Enrollment No</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Course</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Semester</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>Division</v>
+      </c>
+      <c r="G1" t="str">
         <v>Mobile</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>201</v>
+      </c>
+      <c r="B2" t="str">
         <v>999900000001</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Excel Student One</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>B.E.</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>5</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
+        <v>A</v>
+      </c>
+      <c r="G2" t="str">
         <v>9876543212</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>202</v>
+      </c>
+      <c r="B3" t="str">
         <v>999900000002</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Excel Student Two</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>B.E.</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>5</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
+        <v>B</v>
+      </c>
+      <c r="G3" t="str">
         <v>9876543213</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>